<commit_message>
Add historical comparisons and O Grada sensitivity to 1901 account
</commit_message>
<xml_diff>
--- a/ireland-1901/Ireland_1901_BoP_research.xlsx
+++ b/ireland-1901/Ireland_1901_BoP_research.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estimated account" sheetId="1" r:id="Rd38d6403b3e84223"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sandbox" sheetId="2" r:id="R7f070d28fe774f12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Account" sheetId="3" r:id="R2d8e9e9a060d4e8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fiscal comparison" sheetId="4" r:id="R32608a5428c24d31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDP basis" sheetId="5" r:id="R431b0408389e471e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade" sheetId="6" r:id="Rc62c4011d3f04130"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="7" r:id="R65ce5aaf7bba4480"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade inputs" sheetId="8" r:id="R00b61e83162d4ff6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="9" r:id="R3f9280e8e8114e9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Government payments" sheetId="10" r:id="R3c0549ed93f64098"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investment cross-check" sheetId="11" r:id="R90428bdaf7474245"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estate income model" sheetId="12" r:id="R2d2a0869e03147a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Primrose evidence" sheetId="13" r:id="Rf4a922236b414af2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outward property income" sheetId="14" r:id="Rfc76e614c83540b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estimated account" sheetId="1" r:id="Rbc9c6c64b91045d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sandbox" sheetId="2" r:id="R13d96c7ae5de443a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Account" sheetId="3" r:id="Raf3ee59376194afe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fiscal comparison" sheetId="4" r:id="Rd2dced4bf6044b86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDP basis" sheetId="5" r:id="Rd5fd4204b8834841"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade" sheetId="6" r:id="R970a4eccd6d948a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="7" r:id="R61081b19fb284fb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade inputs" sheetId="8" r:id="Rf6cf6b7070d44a65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="9" r:id="R6b2f0dd2735443af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Government payments" sheetId="10" r:id="Rb6eec79f57b44af1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investment cross-check" sheetId="11" r:id="R73cf8fa1c13d47f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estate income model" sheetId="12" r:id="Re6e08f8103354788"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Primrose evidence" sheetId="13" r:id="Rbf89dd1d824c4376"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outward property income" sheetId="14" r:id="R5b6bdcad6977424f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -38,7 +38,7 @@
     <x:numFmt numFmtId="208" formatCode="0.0000"/>
     <x:numFmt numFmtId="209" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="6">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -70,6 +70,11 @@
       <x:sz val="10"/>
       <x:color rgb="FF245AA5"/>
       <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
   <x:fills count="6">
@@ -121,7 +126,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="66">
+  <x:cellXfs count="71">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -307,6 +312,21 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -585,7 +605,7 @@
         <x:v>1900–01</x:v>
       </x:c>
       <x:c r="D7" s="10" t="str">
-        <x:v>Irish services less attributed revenue; Account row 8. Imperial contribution already included.</x:v>
+        <x:v>Irish services less attributed revenue. A fiscal allocation convention, not a complete measure of payments across Ireland’s boundary; see Method rows32–42.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="90" customHeight="1">
@@ -645,7 +665,7 @@
         <x:v>Accepted provisional model</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
-        <x:v>Account B14: company and foreign/colonial government securities.</x:v>
+        <x:v>Accepted estate-model scenario; external institutional earnings remain incomplete. Oldham is not independent validation. See Method rows36–40.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="65" customHeight="1">
@@ -4656,25 +4676,87 @@
       <x:c r="B31" s="2"/>
       <x:c r="C31" s="2"/>
     </x:row>
-    <x:row r="32" ht="23" customHeight="1">
-      <x:c r="A32" s="2"/>
-      <x:c r="B32" s="2"/>
-      <x:c r="C32" s="2"/>
-    </x:row>
-    <x:row r="33" ht="23" customHeight="1">
-      <x:c r="A33" s="2"/>
-      <x:c r="B33" s="2"/>
-      <x:c r="C33" s="2"/>
-    </x:row>
-    <x:row r="34" ht="23" customHeight="1">
-      <x:c r="A34" s="2"/>
-      <x:c r="B34" s="2"/>
-      <x:c r="C34" s="2"/>
-    </x:row>
-    <x:row r="35" ht="23" customHeight="1">
-      <x:c r="A35" s="2"/>
-      <x:c r="B35" s="2"/>
-      <x:c r="C35" s="2"/>
+    <x:row r="32" ht="74" customHeight="1">
+      <x:c r="A32" s="7" t="str">
+        <x:v>Ó Gráda remittance comparison</x:v>
+      </x:c>
+      <x:c r="B32" s="7" t="str">
+        <x:v>£</x:v>
+      </x:c>
+      <x:c r="C32" s="7" t="str">
+        <x:v>Separate substitution in the opening account; ignores mortgage/rent experiments above.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="74" customHeight="1">
+      <x:c r="A33" s="10" t="str">
+        <x:v>All-source remittances to test</x:v>
+      </x:c>
+      <x:c r="B33" s="65" t="n">
+        <x:v>3000000</x:v>
+      </x:c>
+      <x:c r="C33" s="10" t="str">
+        <x:v>Ó Gráda (1994), ch.9, pp.228–229: assumed annual pre-WWI inflow, not a measured 1901 total.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="74" customHeight="1">
+      <x:c r="A34" s="10" t="str">
+        <x:v>Adopted remittances</x:v>
+      </x:c>
+      <x:c r="B34" s="62" t="n">
+        <x:f>'Account'!B18</x:f>
+        <x:v>2054864.8926333094</x:v>
+      </x:c>
+      <x:c r="C34" s="10" t="str">
+        <x:v>Existing US-based proxy; replace this amount, do not add the alternative on top.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="74" customHeight="1">
+      <x:c r="A35" s="10" t="str">
+        <x:v>Change in receipts</x:v>
+      </x:c>
+      <x:c r="B35" s="62" t="n">
+        <x:f>B33-B34</x:f>
+        <x:v>945135.1073666906</x:v>
+      </x:c>
+      <x:c r="C35" s="10" t="str">
+        <x:v>Alternative less adopted remittances.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="74" customHeight="1">
+      <x:c r="A36" s="69" t="str">
+        <x:v>Balance with alternative</x:v>
+      </x:c>
+      <x:c r="B36" s="70" t="n">
+        <x:f>'Estimated account'!B24+B35</x:f>
+        <x:v>-5669737</x:v>
+      </x:c>
+      <x:c r="C36" s="69" t="str">
+        <x:v>Opening estimated account plus change in remittances; other adopted components fixed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="74" customHeight="1">
+      <x:c r="A37" s="48" t="str">
+        <x:v>Income and transfers less rents</x:v>
+      </x:c>
+      <x:c r="B37" s="66" t="n">
+        <x:f>'Estimated account'!B11+'Estimated account'!B12+'Estimated account'!B10+B33+'Estimated account'!B14</x:f>
+        <x:v>450000</x:v>
+      </x:c>
+      <x:c r="C37" s="48" t="str">
+        <x:v>All securities income + seasonal earnings + tested remittances − adopted rents. Includes household UK debt interest, shown as public in the website arrows.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="74" customHeight="1">
+      <x:c r="A38" s="48" t="str">
+        <x:v>Private flow in website arrows</x:v>
+      </x:c>
+      <x:c r="B38" s="66" t="n">
+        <x:f>B37-'Estimated account'!B12</x:f>
+        <x:v>250000</x:v>
+      </x:c>
+      <x:c r="C38" s="48" t="str">
+        <x:v>Previous row less household UK debt interest. Other opening settings held fixed.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -31542,6 +31624,94 @@
       <x:c r="C29" s="2"/>
       <x:c r="D29" s="2"/>
     </x:row>
+    <x:row r="32" ht="30" customHeight="1">
+      <x:c r="A32" s="47" t="str">
+        <x:v>Predecessors and interpretation</x:v>
+      </x:c>
+      <x:c r="B32" s="47" t="str">
+        <x:v>Review of 13 October 2026; adopted figures unchanged.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="115" customHeight="1">
+      <x:c r="A33" s="48" t="str">
+        <x:v>Giffen and the commission</x:v>
+      </x:c>
+      <x:c r="B33" s="48" t="str">
+        <x:v>1896 Financial Relations volume, Lord Farrer and others, printed p.39 / PDF p.43, para.54: approximate exports £25.5m and imports £20m imply £5.5m merchandise surplus. Commissioners question reliability and discuss borrowing, government transfers, absentee payments and emigrant remittances. A contemporary antecedent, not a complete quantified BoP. Original volume-II evidence QQ7621–7630 and appendix pp.174–178 remain to check.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="115" customHeight="1">
+      <x:c r="A34" s="48" t="str">
+        <x:v>Trade revisions</x:v>
+      </x:c>
+      <x:c r="B34" s="48" t="str">
+        <x:v>Oldham, Changes in Irish Exports During Twelve Years (read 1918), pp.541–543, table I: 1904 exports revised from £46,606,432 to £49,212,181 and ultimately £49,784,760. Our commodity sum £49,211,821 differs by £360 from the intermediate control. Retrieve matching revised imports before replacing either side. Continue using 1904 as 1901. https://www.tara.tcd.ie/bitstreams/d9245105-097a-4a50-885e-bebb09092010/download</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="115" customHeight="1">
+      <x:c r="A35" s="48" t="str">
+        <x:v>Fiscal interpretation</x:v>
+      </x:c>
+      <x:c r="B35" s="48" t="str">
+        <x:v>Oldham, The Public Finances of Ireland (1920), pp.15–18: expenditure for Irish services differs from expenditure received in Ireland. Our £2.199m residual is the attributed-revenue-minus-Irish-services convention. Reconcile imperial-service payments to Irish residents and existing £176,000 partial receipts before treating it as a complete external transfer. https://www.tara.tcd.ie/tara8/server/api/core/bitstreams/f69c239e-a144-41d4-b979-11f2d8fdc85d/content</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="115" customHeight="1">
+      <x:c r="A36" s="48" t="str">
+        <x:v>Investment cross-check</x:v>
+      </x:c>
+      <x:c r="B36" s="48" t="str">
+        <x:v>Oldham (1925), The Trade Statistics of the Irish Free State in 1924, pp.118–121, reproduces £949,000 income tax collected and £975,000 attributed for 1900–01. The £26,000 adjustment is tax, not gross investment income. His estate-duty evidence overlaps ours and is not independent validation of £2.2m. https://www.tara.tcd.ie/bitstreams/3e145bed-0076-4ef0-9ac6-9e50254dd506/download</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="115" customHeight="1">
+      <x:c r="A37" s="48" t="str">
+        <x:v>The 1903–04 break</x:v>
+      </x:c>
+      <x:c r="B37" s="48" t="str">
+        <x:v>Primrose, Appendix I, printed p.191 / PDF p.195, records revised allocation based on 1898–99 to 1902–03 estate evidence. Our Primrose evidence tab records the net Irish share changing from 0.2% to 0.7%. Oldham associates the later jump with land purchase, but method changes prevent reading it as measured investment growth.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="115" customHeight="1">
+      <x:c r="A38" s="48" t="str">
+        <x:v>Ó Gráda: remittances</x:v>
+      </x:c>
+      <x:c r="B38" s="48" t="str">
+        <x:v>Cormac Ó Gráda, Ireland: A New Economic History, 1780–1939 (1994), ch.9, pp.228–229: an assumed £3m annual remittance inflow from all sources before WWI. Broader coverage and a later benchmark than our US-based £2.055m proxy. Sandbox rows32–38 show a substitution, not an addition or adoption. Source supplied: Chapter9-151643009.pdf.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="115" customHeight="1">
+      <x:c r="A39" s="48" t="str">
+        <x:v>Ó Gráda: overseas investment</x:v>
+      </x:c>
+      <x:c r="B39" s="48" t="str">
+        <x:v>Ó Gráda (1994), ch.14, p.350: substantial bank savings and London investment; overseas investment need not imply domestic capital scarcity. This directs attention to external institutional earnings, absent from our household securities model. Bank shares held by Irish residents are domestic assets: avoid double-counting their dividends. Source supplied: Chapter14-151643009.pdf.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="115" customHeight="1">
+      <x:c r="A40" s="48" t="str">
+        <x:v>Ó Gráda: integration and convergence</x:v>
+      </x:c>
+      <x:c r="B40" s="48" t="str">
+        <x:v>Ó Gráda (1994), ch.11, p.272: post-Famine convergence in living standards was assisted by migration beyond Britain. Our ownership-income account can coexist with that finding; a net outward flow does not itself establish falling living standards. Source supplied: Chapter11-151643009.pdf.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="115" customHeight="1">
+      <x:c r="A41" s="48" t="str">
+        <x:v>Research positioning</x:v>
+      </x:c>
+      <x:c r="B41" s="48" t="str">
+        <x:v>A reconstruction bringing together and reassessing contemporary estimates for 1901, with explicit assumptions and sensitivity analysis. No claim to be the first Irish BoP. No complete predecessor for precisely all-Ireland 1901 has yet been established in this review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="115" customHeight="1">
+      <x:c r="A42" s="48" t="str">
+        <x:v>Priorities</x:v>
+      </x:c>
+      <x:c r="B42" s="48" t="str">
+        <x:v>Reconcile institutional investment earnings and outward profits; reconcile imperial-service receipts by residence; retrieve paired revised 1904 trade totals. Keep £5m rents and £250,000 seasonal earnings as adopted. Missing flows are omitted, not measured zero; the subtotal does not establish financial-account financing.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Verify Giffen source and retain adopted HNAG trade figures
</commit_message>
<xml_diff>
--- a/ireland-1901/Ireland_1901_BoP_research.xlsx
+++ b/ireland-1901/Ireland_1901_BoP_research.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estimated account" sheetId="1" r:id="Rbc9c6c64b91045d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sandbox" sheetId="2" r:id="R13d96c7ae5de443a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Account" sheetId="3" r:id="Raf3ee59376194afe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fiscal comparison" sheetId="4" r:id="Rd2dced4bf6044b86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDP basis" sheetId="5" r:id="Rd5fd4204b8834841"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade" sheetId="6" r:id="R970a4eccd6d948a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="7" r:id="R61081b19fb284fb3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade inputs" sheetId="8" r:id="Rf6cf6b7070d44a65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="9" r:id="R6b2f0dd2735443af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Government payments" sheetId="10" r:id="Rb6eec79f57b44af1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investment cross-check" sheetId="11" r:id="R73cf8fa1c13d47f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estate income model" sheetId="12" r:id="Re6e08f8103354788"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Primrose evidence" sheetId="13" r:id="Rbf89dd1d824c4376"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outward property income" sheetId="14" r:id="R5b6bdcad6977424f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estimated account" sheetId="1" r:id="R1adae8ac0064439f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sandbox" sheetId="2" r:id="Rfa3f350955d54ec3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Account" sheetId="3" r:id="Rd147257871544899"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fiscal comparison" sheetId="4" r:id="R7c24442e9dcb4294"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDP basis" sheetId="5" r:id="Rac75d1de3a4d460b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade" sheetId="6" r:id="Rae79b5cd46874be5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="7" r:id="Rf58e6d5c8ce842e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade inputs" sheetId="8" r:id="Rc4aa272432094983"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="9" r:id="Rc6c0dea8b7ff4025"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Government payments" sheetId="10" r:id="R3a84c5505cb447fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investment cross-check" sheetId="11" r:id="R0c0112408ade4d92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estate income model" sheetId="12" r:id="Rfc83474e29db4c3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Primrose evidence" sheetId="13" r:id="R47806b00ae2f4ec6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outward property income" sheetId="14" r:id="R750aba910e4c48c1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -31637,7 +31637,7 @@
         <x:v>Giffen and the commission</x:v>
       </x:c>
       <x:c r="B33" s="48" t="str">
-        <x:v>1896 Financial Relations volume, Lord Farrer and others, printed p.39 / PDF p.43, para.54: approximate exports £25.5m and imports £20m imply £5.5m merchandise surplus. Commissioners question reliability and discuss borrowing, government transfers, absentee payments and emigrant remittances. A contemporary antecedent, not a complete quantified BoP. Original volume-II evidence QQ7621–7630 and appendix pp.174–178 remain to check.</x:v>
+        <x:v>Original table verified: C.8008, Second Volume of Minutes of Evidence, printed p.174 / PDF p.414, B.—Supplement to Table III. For 1893: exports £25,574,000; imports £20,054,000; implied surplus £5,520,000. Includes allowances of £1m exports and £2.5m imports for unenumerated goods. Historical comparison only. Kennedy/CEPH/HNAG remains the adopted trade source, with 1904 values used unchanged for 1901. Supplied RoyalCommissionFinancialRelations1896-073783_complete.pdf.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="115" customHeight="1">

</xml_diff>

<commit_message>
Tidy 1901 research workbook and describe its full scope
</commit_message>
<xml_diff>
--- a/ireland-1901/Ireland_1901_BoP_research.xlsx
+++ b/ireland-1901/Ireland_1901_BoP_research.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estimated account" sheetId="1" r:id="R1adae8ac0064439f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sandbox" sheetId="2" r:id="Rfa3f350955d54ec3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Account" sheetId="3" r:id="Rd147257871544899"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fiscal comparison" sheetId="4" r:id="R7c24442e9dcb4294"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDP basis" sheetId="5" r:id="Rac75d1de3a4d460b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade" sheetId="6" r:id="Rae79b5cd46874be5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="7" r:id="Rf58e6d5c8ce842e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade inputs" sheetId="8" r:id="Rc4aa272432094983"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="9" r:id="Rc6c0dea8b7ff4025"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Government payments" sheetId="10" r:id="R3a84c5505cb447fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investment cross-check" sheetId="11" r:id="R0c0112408ade4d92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estate income model" sheetId="12" r:id="Rfc83474e29db4c3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Primrose evidence" sheetId="13" r:id="R47806b00ae2f4ec6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outward property income" sheetId="14" r:id="R750aba910e4c48c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estimated account" sheetId="1" r:id="R539ad8efcac84c33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sandbox" sheetId="2" r:id="Rb3bd718237b6429b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Account" sheetId="3" r:id="Rac2ca687c7134cee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fiscal comparison" sheetId="4" r:id="R9d72eb023725492a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDP basis" sheetId="5" r:id="Rf83f45cf3fa14921"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade" sheetId="6" r:id="R375d27c2f9b0413d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="7" r:id="Rc42aabcb92474875"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade inputs" sheetId="8" r:id="Rd31dfb69038d432b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="9" r:id="Rdd20b7dafde64ab2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Government payments" sheetId="10" r:id="R0ecb97db088e411a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investment cross-check" sheetId="11" r:id="R7eed825a41dd4edc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estate income model" sheetId="12" r:id="R0f289ffe470e458e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Primrose evidence" sheetId="13" r:id="R5389db7e528640e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outward property income" sheetId="14" r:id="Rcdb39cc492b74a8b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -550,9 +550,9 @@
       <x:c r="C2" s="2"/>
       <x:c r="D2" s="2"/>
     </x:row>
-    <x:row r="3" ht="38" customHeight="1">
+    <x:row r="3" ht="42" customHeight="1">
       <x:c r="A3" s="60" t="str">
-        <x:v>Working estimate: positive = receipts; negative = payments. Existing Account retains previously adopted entries and evidence status.</x:v>
+        <x:v>Start here: the opening estimate for all-Ireland, circa 1901. Annual £; receipts positive, payments negative. Sources and assumptions are listed beside each component.</x:v>
       </x:c>
       <x:c r="B3" s="60"/>
       <x:c r="C3" s="60"/>
@@ -578,7 +578,7 @@
         <x:v>Source / assumption</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="65" customHeight="1">
+    <x:row r="6" ht="48" customHeight="1">
       <x:c r="A6" s="10" t="str">
         <x:v>Merchandise trade</x:v>
       </x:c>
@@ -587,13 +587,13 @@
         <x:v>-4096737</x:v>
       </x:c>
       <x:c r="C6" s="10" t="str">
-        <x:v>Agreed proxy</x:v>
+        <x:v>Source-year proxy</x:v>
       </x:c>
       <x:c r="D6" s="10" t="str">
-        <x:v>1904 values used unchanged for 1901; Account row 7 / Trade.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="65" customHeight="1">
+        <x:v>Kennedy / CEPH / HNAG: 1904 merchandise values used unchanged for 1901.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="48" customHeight="1">
       <x:c r="A7" s="10" t="str">
         <x:v>Fiscal residual</x:v>
       </x:c>
@@ -605,10 +605,10 @@
         <x:v>1900–01</x:v>
       </x:c>
       <x:c r="D7" s="10" t="str">
-        <x:v>Irish services less attributed revenue. A fiscal allocation convention, not a complete measure of payments across Ireland’s boundary; see Method rows32–42.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="90" customHeight="1">
+        <x:v>Irish services less attributed revenue. Territorial allocation, not a complete cash-flow measure; see Method.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="48" customHeight="1">
       <x:c r="A8" s="10" t="str">
         <x:v>Army works: local receipts proxy</x:v>
       </x:c>
@@ -620,10 +620,10 @@
         <x:v>Partial spending proxy</x:v>
       </x:c>
       <x:c r="D8" s="10" t="str">
-        <x:v>Government payments B5. Assume selected expenditure reaches Irish residents; residency and merchandise overlap not yet reconciled. Rounded to £10,000; not total military expenditure.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="90" customHeight="1">
+        <x:v>Selected Army works, rounded. Recipient residence and overlap with trade remain unresolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="48" customHeight="1">
       <x:c r="A9" s="10" t="str">
         <x:v>Kilmainham Hospital spending</x:v>
       </x:c>
@@ -635,10 +635,10 @@
         <x:v>Partial spending proxy</x:v>
       </x:c>
       <x:c r="D9" s="10" t="str">
-        <x:v>Government payments B6. Assume local receipts outside Irish-services fiscal total; pending reconciliation. Institutional spending, not a separate household pension estimate.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="65" customHeight="1">
+        <x:v>Institutional spending outside the Irish-services total, subject to overlap checks.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="48" customHeight="1">
       <x:c r="A10" s="10" t="str">
         <x:v>Seasonal workers</x:v>
       </x:c>
@@ -647,13 +647,13 @@
         <x:v>250000</x:v>
       </x:c>
       <x:c r="C10" s="10" t="str">
-        <x:v>Agreed estimate</x:v>
+        <x:v>Rounded estimate</x:v>
       </x:c>
       <x:c r="D10" s="10" t="str">
-        <x:v>£250,000 rounded net earnings brought home; Account B13.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="65" customHeight="1">
+        <x:v>Rounded net earnings brought home; 1901 Migratory Labourers report and regional evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="48" customHeight="1">
       <x:c r="A11" s="10" t="str">
         <x:v>Other overseas securities income</x:v>
       </x:c>
@@ -662,13 +662,13 @@
         <x:v>2000000</x:v>
       </x:c>
       <x:c r="C11" s="10" t="str">
-        <x:v>Accepted provisional model</x:v>
+        <x:v>Provisional model</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
-        <x:v>Accepted estate-model scenario; external institutional earnings remain incomplete. Oldham is not independent validation. See Method rows36–40.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="65" customHeight="1">
+        <x:v>Estate model: company and foreign-government securities. Institutional overseas earnings remain incomplete.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="48" customHeight="1">
       <x:c r="A12" s="10" t="str">
         <x:v>UK public debt: household income</x:v>
       </x:c>
@@ -677,13 +677,13 @@
         <x:v>200000</x:v>
       </x:c>
       <x:c r="C12" s="10" t="str">
-        <x:v>Accepted provisional model</x:v>
+        <x:v>Provisional model</x:v>
       </x:c>
       <x:c r="D12" s="10" t="str">
-        <x:v>Account B16: £200,000 from estate model.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="90" customHeight="1">
+        <x:v>Estate model: direct household holdings of UK public debt.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="48" customHeight="1">
       <x:c r="A13" s="10" t="str">
         <x:v>Bank of Ireland: UK debt interest</x:v>
       </x:c>
@@ -695,10 +695,10 @@
         <x:v>Contractual proxy</x:v>
       </x:c>
       <x:c r="D13" s="10" t="str">
-        <x:v>Government payments B8, rounded to £10,000. Treat as institutional receipt additional to household direct UK debt holdings; verify 1901 receipt. Do not also classify Irish bank shares as external holdings.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="65" customHeight="1">
+        <x:v>Rounded contractual interest. Separate from household holdings; actual 1901 receipt remains to verify.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="48" customHeight="1">
       <x:c r="A14" s="10" t="str">
         <x:v>Absentee rents</x:v>
       </x:c>
@@ -710,10 +710,10 @@
         <x:v>Selected 1895 proxy</x:v>
       </x:c>
       <x:c r="D14" s="10" t="str">
-        <x:v>Account B15: £5m; older £3.46m retained in sensitivity.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="90" customHeight="1">
+        <x:v>O’Brien (1895), £5m. The older £3.46m alternative is available in Sandbox.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="48" customHeight="1">
       <x:c r="A15" s="10" t="str">
         <x:v>Additional mortgage interest</x:v>
       </x:c>
@@ -724,10 +724,10 @@
         <x:v>Unresolved overlap</x:v>
       </x:c>
       <x:c r="D15" s="10" t="str">
-        <x:v>£630,000 historical interest is available, but its addition to rents is unmeasured. Scenario experiments are on Sandbox and do not feed this subtotal.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="65" customHeight="1">
+        <x:v>Historical £630,000 interest estimate; overlap with rents unresolved. Test separately in Sandbox.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="48" customHeight="1">
       <x:c r="A16" s="10" t="str">
         <x:v>Emigrant remittances</x:v>
       </x:c>
@@ -736,13 +736,13 @@
         <x:v>2054864.8926333094</x:v>
       </x:c>
       <x:c r="C16" s="10" t="str">
-        <x:v>Agreed proxy</x:v>
+        <x:v>Source-year proxy</x:v>
       </x:c>
       <x:c r="D16" s="10" t="str">
-        <x:v>Account B18: US estimate adopted, with no extra bank/postal addition.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="65" customHeight="1">
+        <x:v>US remittances of $10m (1906), converted at $4.8665/£. Bank and postal components already included.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="48" customHeight="1">
       <x:c r="A17" s="10" t="str">
         <x:v>Shipping / passenger transport</x:v>
       </x:c>
@@ -753,10 +753,10 @@
         <x:v>No usable estimate yet</x:v>
       </x:c>
       <x:c r="D17" s="10" t="str">
-        <x:v>Needs resident carrier receipts and payments plus trade valuation reconciliation.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="65" customHeight="1">
+        <x:v>Resident carrier earnings and payments; reconcile freight in merchandise values.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="48" customHeight="1">
       <x:c r="A18" s="10" t="str">
         <x:v>Insurance / other business services</x:v>
       </x:c>
@@ -767,10 +767,10 @@
         <x:v>No usable estimate yet</x:v>
       </x:c>
       <x:c r="D18" s="10" t="str">
-        <x:v>Premiums are not equivalent to service charges.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="65" customHeight="1">
+        <x:v>Service charges require estimation; gross premiums are not the service flow.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="48" customHeight="1">
       <x:c r="A19" s="10" t="str">
         <x:v>Tourism / travel</x:v>
       </x:c>
@@ -781,10 +781,10 @@
         <x:v>No usable estimate yet</x:v>
       </x:c>
       <x:c r="D19" s="10" t="str">
-        <x:v>Both directions; avoid worker-expense duplication.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="65" customHeight="1">
+        <x:v>Receipts and spending in both directions; exclude seasonal-worker expenses already deducted.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="48" customHeight="1">
       <x:c r="A20" s="10" t="str">
         <x:v>Other company-profit outflows</x:v>
       </x:c>
@@ -795,10 +795,10 @@
         <x:v>No usable estimate yet</x:v>
       </x:c>
       <x:c r="D20" s="10" t="str">
-        <x:v>Includes Guinness ownership question; distinct from absentee rent.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="65" customHeight="1">
+        <x:v>External ownership of Irish businesses, including Guinness, remains unmeasured.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="48" customHeight="1">
       <x:c r="A21" s="10" t="str">
         <x:v>Additional external pensions</x:v>
       </x:c>
@@ -809,10 +809,10 @@
         <x:v>No usable estimate yet</x:v>
       </x:c>
       <x:c r="D21" s="10" t="str">
-        <x:v>Superannuation already in fiscal residual; hospital proxy separately above.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="65" customHeight="1">
+        <x:v>Further overseas pensions only; superannuation already included in Irish services.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="48" customHeight="1">
       <x:c r="A22" s="10" t="str">
         <x:v>Other current transfers</x:v>
       </x:c>
@@ -823,7 +823,7 @@
         <x:v>No usable estimate yet</x:v>
       </x:c>
       <x:c r="D22" s="10" t="str">
-        <x:v>No quantitative basis yet.</x:v>
+        <x:v>Other cross-border current transfers remain unmeasured.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="65" customHeight="1">
@@ -832,7 +832,7 @@
       <x:c r="C23" s="10"/>
       <x:c r="D23" s="10"/>
     </x:row>
-    <x:row r="24" ht="65" customHeight="1">
+    <x:row r="24" ht="40" customHeight="1">
       <x:c r="A24" s="10" t="str">
         <x:v>Working subtotal, estimated items</x:v>
       </x:c>
@@ -847,7 +847,7 @@
         <x:v>Text entries above are omitted from the sum, not assumed to be measured zero.</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="65" customHeight="1">
+    <x:row r="25" ht="40" customHeight="1">
       <x:c r="A25" s="22" t="str">
         <x:v>Reported subtotal, rounded</x:v>
       </x:c>
@@ -874,14 +874,14 @@
       <x:c r="C27" s="10"/>
       <x:c r="D27" s="10"/>
     </x:row>
-    <x:row r="28" ht="80" customHeight="1">
+    <x:row r="28" ht="56" customHeight="1">
       <x:c r="A28" s="7" t="str">
         <x:v>Experiment separately</x:v>
       </x:c>
       <x:c r="B28" s="7"/>
       <x:c r="C28" s="7"/>
       <x:c r="D28" s="7" t="str">
-        <x:v>Use the Sandbox tab to change rents and mortgage assumptions. Sandbox changes never alter this working account. This account retains the previously accepted provisional income scenario and partial spending proxies.</x:v>
+        <x:v>Sandbox tests alternatives without changing this estimate. Account holds component inputs; the remaining tabs contain calculations, original evidence and source references.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="90" customHeight="1">
@@ -2542,12 +2542,12 @@
     </x:row>
     <x:row r="20" ht="65" customHeight="1">
       <x:c r="A20" s="10" t="str">
-        <x:v>Next source check</x:v>
+        <x:v>Tax adjustment verified</x:v>
       </x:c>
       <x:c r="B20" s="2"/>
       <x:c r="C20" s="2"/>
       <x:c r="D20" s="10" t="str">
-        <x:v>Original 1900–01 true-revenue adjustment now verified below. It reallocates tax receipts, not gross investment income; the gross-income calculation above remains a separate provisional cross-check.</x:v>
+        <x:v>Rows35–45 verify the 1900–01 tax allocation. It is not gross investment income; the calculation above is a separate cross-check.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="48" customHeight="1">
@@ -3091,7 +3091,7 @@
     </x:row>
     <x:row r="4" ht="23" customHeight="1">
       <x:c r="A4" s="10" t="str">
-        <x:v>1901 reconstruction — provisional working scenario accepted by user</x:v>
+        <x:v>1901 reconstruction: provisional estate-income model</x:v>
       </x:c>
       <x:c r="B4" s="10"/>
       <x:c r="C4" s="10"/>
@@ -3668,7 +3668,7 @@
     </x:row>
     <x:row r="46" ht="82" customHeight="1">
       <x:c r="A46" s="10" t="str">
-        <x:v>Primrose source obtained</x:v>
+        <x:v>Primrose evidence</x:v>
       </x:c>
       <x:c r="B46" s="10"/>
       <x:c r="C46" s="10"/>
@@ -3689,7 +3689,7 @@
       <x:c r="E47" s="10"/>
       <x:c r="F47" s="10"/>
       <x:c r="G47" s="10" t="str">
-        <x:v>User accepted £2.2m as provisional working estimate on 13 October 2026. Account splits rounded amounts between other overseas securities (£2.0m) and UK public debt (£0.2m). Assumptions and sensitivity remain explicit; not a verified estimate.</x:v>
+        <x:v>Rounded working estimate £2.2m: £2m other overseas securities and £0.2m UK public debt. Portfolio shares, yields and the estate multiplier remain assumptions.</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="23" customHeight="1">
@@ -4041,10 +4041,10 @@
         <x:v>Decision for reconstruction</x:v>
       </x:c>
       <x:c r="B17" s="10" t="str">
-        <x:v>Provisional scenario accepted</x:v>
+        <x:v>Provisional working model</x:v>
       </x:c>
       <x:c r="C17" s="10" t="str">
-        <x:v>User accepted estate-income working scenario on 13 October 2026. Primrose improves interpretation but does not resolve issuer split, mortality multiplier or yields. No separate Guinness estimate has yet been made.</x:v>
+        <x:v>Primrose clarifies interpretation but does not resolve the issuer split, estate multiplier or yields. Guinness has not been estimated separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="23" customHeight="1">
@@ -4182,7 +4182,7 @@
         <x:v>5000000</x:v>
       </x:c>
       <x:c r="C9" s="10" t="str">
-        <x:v>1895 memorandum: probable amount covering rental rows 1–3. User-selected provisional main estimate for 1901 because it is closer in date. Contemporary judgment, not a fresh census or observed remittance total.</x:v>
+        <x:v>1895 memorandum: probable amount covering rental rows 1–3. Provisional main estimate for 1901 because it is closer in date. Contemporary judgment, not a fresh census or observed remittance total.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="88" customHeight="1">
@@ -4348,7 +4348,7 @@
       </x:c>
       <x:c r="B27" s="10"/>
       <x:c r="C27" s="10" t="str">
-        <x:v>User prioritises the closer-date estimate: £5m absentee rents entered provisionally in Account. £3.46m remains an alternative, not a confidence bound. No separate mortgage addition or unsupported land-purchase adjustment.</x:v>
+        <x:v>Closer-date working estimate: £5m absentee rents entered provisionally in Account. £3.46m remains an alternative, not a confidence bound. No separate mortgage addition or unsupported land-purchase adjustment.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="23" customHeight="1">
@@ -4488,7 +4488,7 @@
         <x:v>5000000</x:v>
       </x:c>
       <x:c r="C10" s="10" t="str">
-        <x:v>Default is user-selected £5m. Older-evidence comparison £3,461,716. Positive outward amount.</x:v>
+        <x:v>Opening estimate £5m; older comparison £3,461,716. Positive outward amount.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="72" customHeight="1">
@@ -4791,7 +4791,7 @@
     </x:row>
     <x:row r="2" ht="23" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>Ireland balance of payments, circa 1901</x:v>
+        <x:v>Component ledger: inputs to the opening estimate</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -4807,9 +4807,9 @@
       <x:c r="E3" s="4"/>
       <x:c r="F3" s="4"/>
     </x:row>
-    <x:row r="4" ht="23" customHeight="1">
+    <x:row r="4" ht="42" customHeight="1">
       <x:c r="A4" s="2" t="str">
-        <x:v>All-island Ireland. Sterling. Credits positive; debits negative. First research assembly, 11 October 2026.</x:v>
+        <x:v>Supporting inputs, not a second headline estimate. Estimated account adds the partial public receipts. Annual £; all-Ireland; receipts positive and payments negative.</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -4960,7 +4960,7 @@
       </x:c>
       <x:c r="E13" s="2"/>
       <x:c r="F13" s="10" t="str">
-        <x:v>User-adopted all-Ireland working estimate: £250,000 net earnings brought home. Migratory labourers report for 1901 and earlier regional evidence; rounding is deliberate. Do not add gross earnings without deducting overseas expenses.</x:v>
+        <x:v>All-Ireland working estimate: £250,000 net earnings brought home. Migratory labourers report for 1901 and earlier regional evidence; rounding is deliberate. Do not add gross earnings without deducting overseas expenses.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="50" customHeight="1">
@@ -4979,7 +4979,7 @@
       </x:c>
       <x:c r="E14" s="2"/>
       <x:c r="F14" s="10" t="str">
-        <x:v>User accepts provisional scenario. Company securities plus foreign/colonial government securities, rounded to £100,000. 50% external company share and illustrative yields remain unverified. UK public debt is separately in row 16. No company-specific Guinness adjustment has been estimated.</x:v>
+        <x:v>Provisional scenario. Company securities plus foreign/colonial government securities, rounded to £100,000. 50% external company share and illustrative yields remain unverified. UK public debt is separately in row 16. No company-specific Guinness adjustment has been estimated.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="50" customHeight="1">
@@ -4998,7 +4998,7 @@
       </x:c>
       <x:c r="E15" s="2"/>
       <x:c r="F15" s="10" t="str">
-        <x:v>User prioritises O’Brien’s £5m probable rental estimate presented in 1895. Retain £3.46m older-evidence alternative in Outward property income. No measured 1895–1901 adjustment; additional mortgage interest and company profits remain unmeasured, not zero.</x:v>
+        <x:v>The adopted estimate uses O’Brien’s £5m probable rental estimate presented in 1895. Retain £3.46m older-evidence alternative in Outward property income. No measured 1895–1901 adjustment; additional mortgage interest and company profits remain unmeasured, not zero.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="50" customHeight="1">
@@ -5052,7 +5052,7 @@
       </x:c>
       <x:c r="E18" s="2"/>
       <x:c r="F18" s="10" t="str">
-        <x:v>User adopts E20 as working remittance receipts. US inflow, no additional GB uplift. Source bank and postal components are included, not added again.</x:v>
+        <x:v>E20 supplies working remittance receipts. US inflow, no additional GB uplift. Source bank and postal components are included, not added again.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="50" customHeight="1">
@@ -5089,7 +5089,7 @@
       </x:c>
       <x:c r="C21" s="22"/>
       <x:c r="D21" s="22" t="str">
-        <x:v>Incomplete: not a current-account total</x:v>
+        <x:v>Excludes partial public receipts; see Estimated account</x:v>
       </x:c>
       <x:c r="E21" s="2"/>
       <x:c r="F21" s="10"/>
@@ -7015,7 +7015,7 @@
       </x:c>
       <x:c r="D15" s="2"/>
       <x:c r="E15" s="10" t="str">
-        <x:v>Working assumption agreed 11 October 2026: use the HNAG 1904 values unchanged as proxies for 1901. No price or quantity adjustment. Source year remains 1904.</x:v>
+        <x:v>Working assumption: use the HNAG 1904 values unchanged as proxies for 1901. No price or quantity adjustment. Source year remains 1904.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="23" customHeight="1">
@@ -7756,7 +7756,7 @@
         <x:v>Approximate contemporary estimate</x:v>
       </x:c>
       <x:c r="G24" s="10" t="str">
-        <x:v>Adopted unchanged as working 1901 remittance proxy, user instruction 11 October 2026.</x:v>
+        <x:v>Adopted unchanged as working 1901 remittance proxy, source-year proxy.</x:v>
       </x:c>
       <x:c r="H24" s="2"/>
       <x:c r="I24" s="10" t="str">
@@ -8004,7 +8004,7 @@
       </x:c>
       <x:c r="H33" s="2"/>
       <x:c r="I33" s="10" t="str">
-        <x:v>E20 / E28. User adoption 11 October 2026. https://fraser.stlouisfed.org/title/credit-nations-trade-balance-united-states-620/fulltext</x:v>
+        <x:v>E20 / E28. https://fraser.stlouisfed.org/title/credit-nations-trade-balance-united-states-620/fulltext</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="23" customHeight="1">
@@ -31366,220 +31366,220 @@
         <x:v>Source / next record to obtain</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="80" customHeight="1">
+    <x:row r="5" ht="64" customHeight="1">
       <x:c r="A5" s="10" t="str">
-        <x:v>1822 model</x:v>
+        <x:v>Scope</x:v>
       </x:c>
       <x:c r="B5" s="10" t="str">
-        <x:v>Retain merchandise, public and private flows, source-based alternatives, resident-recipient adjustments, and a partial residual. Extend services, labour income, remittances and financing. Do not carry 1822 values or assumed allocation percentages into 1901.</x:v>
+        <x:v>All-Ireland circa 1901; Great Britain counts as overseas. Annual sterling flows. Source-year substitutions are identified.</x:v>
       </x:c>
       <x:c r="C5" s="2"/>
       <x:c r="D5" s="10" t="str">
         <x:v>https://chris-colvin.github.io/ireland-1822.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="80" customHeight="1">
+    <x:row r="6" ht="64" customHeight="1">
       <x:c r="A6" s="10" t="str">
-        <x:v>Origin of the fiscal return</x:v>
+        <x:v>Fiscal return</x:v>
       </x:c>
       <x:c r="B6" s="10" t="str">
-        <x:v>Oldham traces the return to Goschen’s 1890 inquiry, publication as Parliamentary Paper 329 (1891), and revision as Paper 93 (1893) for the Home Rule debates. This is the origin of the comparative return, not the first use of the term Imperial contribution.</x:v>
+        <x:v>The comparative return began in 1891, following Goschen’s inquiry, and was revised in 1893. This dates the return, not the term “imperial contribution”.</x:v>
       </x:c>
       <x:c r="C6" s="2"/>
       <x:c r="D6" s="10" t="str">
         <x:v>https://www.tara.tcd.ie/tara8/server/api/core/bitstreams/f69c239e-a144-41d4-b979-11f2d8fdc85d/content</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="80" customHeight="1">
+    <x:row r="7" ht="64" customHeight="1">
       <x:c r="A7" s="10" t="str">
-        <x:v>Union quota and 1817</x:v>
+        <x:v>Union and 1817</x:v>
       </x:c>
       <x:c r="B7" s="10" t="str">
-        <x:v>Article VII prescribed GB:Ireland contributions of 15:2. Exchequer amalgamation in 1817 ended the fixed quota. The 1822 territorial accounts and 1901 Irish-services classification are not directly comparable.</x:v>
+        <x:v>The Union’s 15:2 contribution quota ended with exchequer amalgamation in 1817. The 1822 and 1901 territorial classifications differ.</x:v>
       </x:c>
       <x:c r="C7" s="2"/>
       <x:c r="D7" s="10" t="str">
         <x:v>https://en.wikisource.org/wiki/Act_of_Union_1800 ; https://www.gutenberg.org/files/15086/15086-h/15086-h.htm</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="80" customHeight="1">
+    <x:row r="8" ht="64" customHeight="1">
       <x:c r="A8" s="10" t="str">
-        <x:v>Fiscal subtotal</x:v>
+        <x:v>Fiscal treatment</x:v>
       </x:c>
       <x:c r="B8" s="10" t="str">
-        <x:v>Attributed revenue less domestic services is an accounting residual. For external flows establish tax incidence, recipient residence and any government purchases already counted in trade. Benefits of spending are a separate question.</x:v>
+        <x:v>Attributed revenue less Irish services is an allocation residual. Recipient residence and procurement overlap remain to reconcile.</x:v>
       </x:c>
       <x:c r="C8" s="2"/>
       <x:c r="D8" s="10" t="str">
         <x:v>https://en.wikisource.org/wiki/Problems_of_Empire/The_Finance_of_Federal_Government_for_the_United_Kingdom#APPENDIX.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="80" customHeight="1">
+    <x:row r="9" ht="64" customHeight="1">
       <x:c r="A9" s="10" t="str">
-        <x:v>Fiscal source discrepancy</x:v>
+        <x:v>Irish fiscal sources</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>Brassey gives Irish revenue £9.505m, Scotfact £9.521m. Hansard gives services £7.268m, versus £7.306m in HNAG and Brassey. Preserve all versions. Obtain original return 90 (1901) and the return behind HNAG’s 1902 LV citation.</x:v>
+        <x:v>The original 1900–01 return is available. Adopted revenue £9.505m and services £7.306m; alternative transcriptions are retained in Fiscal comparison.</x:v>
       </x:c>
       <x:c r="C9" s="2"/>
       <x:c r="D9" s="10" t="str">
-        <x:v>https://api.parliament.uk/historic-hansard/commons/1901/jul/18/financial-relations-of-great-britain-and ; https://www.scotfact.com/article_scotland20thCentury_data</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="80" customHeight="1">
+        <x:v>RevenueAndExpenditure1901-000393_complete.pdf, printed pp.6–7 / PDF pp.18–19; Fiscal comparison.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="64" customHeight="1">
       <x:c r="A10" s="10" t="str">
-        <x:v>England transcription discrepancy</x:v>
+        <x:v>British fiscal sources</x:v>
       </x:c>
       <x:c r="B10" s="10" t="str">
-        <x:v>Brassey’s opening summary gives revenue £113.244m; Table V transcription gives £113.224m. The opening value equals services £34.769m plus contribution £78.475m and reconciles the total. Adopt it explicitly pending scan verification.</x:v>
+        <x:v>England’s £113.244m revenue reconciles to services plus contribution. Brassey’s £113.224m alternative is retained as a transcription discrepancy.</x:v>
       </x:c>
       <x:c r="C10" s="2"/>
       <x:c r="D10" s="10" t="str">
         <x:v>https://en.wikisource.org/wiki/Problems_of_Empire/The_Finance_of_Federal_Government_for_the_United_Kingdom#APPENDIX.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="80" customHeight="1">
+    <x:row r="11" ht="64" customHeight="1">
       <x:c r="A11" s="10" t="str">
-        <x:v>GDP denominator</x:v>
+        <x:v>Output denominators</x:v>
       </x:c>
       <x:c r="B11" s="10" t="str">
-        <x:v>Use matched Millennium v3.1 current factor-cost output for Ireland, GB and UK. The workbook cites Andersson–Lennard (2017); the final paper has a different real growth path. Preserve older estimates and the price-base/vintage audit on GDP basis.</x:v>
+        <x:v>Matched Millennium v3.1 current factor-cost estimates for Ireland, GB and UK. GDP basis records the Andersson–Lennard reference, vintage differences and older estimates.</x:v>
       </x:c>
       <x:c r="C11" s="2"/>
       <x:c r="D11" s="10" t="str">
         <x:v>https://www.bankofengland.co.uk/-/media/boe/files/statistics/research-datasets/a-millennium-of-macroeconomic-data-for-the-uk.xlsx ; https://doi.org/10.1093/ereh/hey003</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="80" customHeight="1">
+    <x:row r="12" ht="64" customHeight="1">
       <x:c r="A12" s="10" t="str">
-        <x:v>Trade proxy adopted</x:v>
+        <x:v>Trade</x:v>
       </x:c>
       <x:c r="B12" s="10" t="str">
-        <x:v>Use HNAG 1904 exports and imports unchanged for 1901, agreed 11 October 2026. Backcasting is deferred. Preserve the £360 export control discrepancy and matched report vintage. Next priority is actual public receipts.</x:v>
+        <x:v>Kennedy / CEPH / HNAG 1904 values used unchanged for 1901. Trade retains the £360 control discrepancy and later export revision; adopted figures are unchanged.</x:v>
       </x:c>
       <x:c r="C12" s="2"/>
       <x:c r="D12" s="10" t="str">
         <x:v>https://ceph.ie/data-set/international-trade/ ; https://www.tara.tcd.ie/bitstreams/28069c61-813a-4e79-8e67-9ddc49b205dc/download ; https://www.tara.tcd.ie/bitstreams/d9245105-097a-4a50-885e-bebb09092010/download</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="80" customHeight="1">
+    <x:row r="13" ht="64" customHeight="1">
       <x:c r="A13" s="10" t="str">
-        <x:v>Priority 2: actual public receipts</x:v>
+        <x:v>Public receipts</x:v>
       </x:c>
       <x:c r="B13" s="10" t="str">
-        <x:v>Find territorial Army/Navy expenditure, pensions and debt interest around 1900–01. Separate locally received pay and purchases from headquarters charges. Identify procurement already captured as exports.</x:v>
+        <x:v>Selected works, hospital spending and interest are provisional additions. Further military and naval receipts require evidence of recipient residence and overlap.</x:v>
       </x:c>
       <x:c r="C13" s="2"/>
       <x:c r="D13" s="10" t="str">
         <x:v>Parliamentary Army and Navy accounts, geographical expenditure returns, and Treasury papers. No usable 1901 total yet located.</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="80" customHeight="1">
+    <x:row r="14" ht="64" customHeight="1">
       <x:c r="A14" s="10" t="str">
-        <x:v>Priority 3: seasonal earnings</x:v>
+        <x:v>Seasonal earnings</x:v>
       </x:c>
       <x:c r="B14" s="10" t="str">
-        <x:v>Get Report, Maps and Appendices relating to Migratory Irish Agricultural Labourers (Cd.341, 1900) and the 1901 continuation. Wilson Fox has actual 1901 farm earnings examples but cautions against aggregation across unlike employment periods.</x:v>
+        <x:v>£250,000 net earnings brought home, rounded from the 1901 report and regional evidence. The report has been obtained.</x:v>
       </x:c>
       <x:c r="C14" s="2"/>
       <x:c r="D14" s="10" t="str">
-        <x:v>https://ceph.ie/wp-content/uploads/2024/04/Wilson-Fox.pdf ; https://hansard.parliament.uk/%E2%80%8CCommons/1902-01-24/debates/49b63972-856a-4bef-a90d-2352cf8ff887/IrishLandQuestion</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="80" customHeight="1">
+        <x:v>1902-001933_complete-MigratoryLabourers1901.pdf; regional evidence: https://hansard.parliament.uk/%E2%80%8CCommons/1902-01-24/debates/49b63972-856a-4bef-a90d-2352cf8ff887/IrishLandQuestion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="64" customHeight="1">
       <x:c r="A15" s="10" t="str">
-        <x:v>Seasonal migration counts</x:v>
+        <x:v>Migration counts</x:v>
       </x:c>
       <x:c r="B15" s="10" t="str">
-        <x:v>1904 home enumeration gives 17,589, including 7.8% migrating within Ireland; transport records give 33,470 with repeat trips. Do not treat journeys as unique workers or sum overlapping counts.</x:v>
+        <x:v>Enumeration and transport counts differ: journeys can include repeat trips and migration within Ireland. They are not interchangeable worker totals.</x:v>
       </x:c>
       <x:c r="C15" s="2"/>
       <x:c r="D15" s="10" t="str">
         <x:v>https://ceph.ie/wp-content/uploads/2024/04/Wilson-Fox.pdf</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="80" customHeight="1">
+    <x:row r="16" ht="64" customHeight="1">
       <x:c r="A16" s="10" t="str">
-        <x:v>Remittances adopted</x:v>
+        <x:v>Remittances</x:v>
       </x:c>
       <x:c r="B16" s="10" t="str">
-        <x:v>Use the approximately $10m US-to-Ireland figure for 1906 unchanged as the working 1901 remittance receipts estimate, agreed 11 October 2026. Convert at $4.8665 per pound. No additional GB uplift. This is a receipt proxy, not a measured net transfer balance.</x:v>
+        <x:v>US estimate of $10m for 1906 used for 1901 at $4.8665/£. No additional GB uplift. Ó Gráda’s all-source alternative is tested in Sandbox.</x:v>
       </x:c>
       <x:c r="C16" s="2"/>
       <x:c r="D16" s="10" t="str">
         <x:v>https://fraser.stlouisfed.org/title/credit-nations-trade-balance-united-states-620/fulltext</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="80" customHeight="1">
+    <x:row r="17" ht="64" customHeight="1">
       <x:c r="A17" s="10" t="str">
-        <x:v>Priority 5: private income</x:v>
+        <x:v>Investment income</x:v>
       </x:c>
       <x:c r="B17" s="10" t="str">
-        <x:v>Use HNAG income-tax schedules C and D as leads, with resident ownership evidence for rents, mortgages, railway and company securities, bank assets and foreign investments. Income-tax geography is not creditor residence.</x:v>
+        <x:v>£2.2m provisional estate model. Tax-assessment location does not establish residence of owners or issuers. Institutional earnings and outward company profits remain incomplete.</x:v>
       </x:c>
       <x:c r="C17" s="2"/>
       <x:c r="D17" s="10" t="str">
         <x:v>https://ceph.ie/data-set/public-finance/</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="80" customHeight="1">
+    <x:row r="18" ht="64" customHeight="1">
       <x:c r="A18" s="10" t="str">
-        <x:v>Priority 6: transport and insurance</x:v>
+        <x:v>Transport and insurance</x:v>
       </x:c>
       <x:c r="B18" s="10" t="str">
-        <x:v>Read trade valuation notes, shipping-company accounts and Board of Trade returns. Ships built and sold are goods; their operating earnings are services. Registered tonnage alone cannot establish net earnings.</x:v>
+        <x:v>Not yet estimated. Reconcile transport in trade values; ships sold are goods, operating earnings are services.</x:v>
       </x:c>
       <x:c r="C18" s="2"/>
       <x:c r="D18" s="10" t="str">
         <x:v>Trade reports and company accounts; no defensible aggregate yet adopted.</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="80" customHeight="1">
+    <x:row r="19" ht="64" customHeight="1">
       <x:c r="A19" s="10" t="str">
-        <x:v>Priority 7: travel</x:v>
+        <x:v>Travel</x:v>
       </x:c>
       <x:c r="B19" s="10" t="str">
-        <x:v>Find passenger counts, tourist surveys or contemporary spending estimates. Separate visitors, emigrants, seasonal workers and Irish residents returning from travel.</x:v>
+        <x:v>Not yet estimated. Separate tourists, emigrants and seasonal workers to avoid duplication.</x:v>
       </x:c>
       <x:c r="C19" s="2"/>
       <x:c r="D19" s="10" t="str">
         <x:v>Railway and steamship records; no defensible aggregate yet adopted.</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="80" customHeight="1">
+    <x:row r="20" ht="64" customHeight="1">
       <x:c r="A20" s="10" t="str">
         <x:v>Financing</x:v>
       </x:c>
       <x:c r="B20" s="10" t="str">
-        <x:v>Investigate land-purchase advances, principal repayments, securities transactions and bank external assets/liabilities. Income is current; principal is financial. Bank deposits at home do not by themselves measure external flows.</x:v>
+        <x:v>Principal movements, land-purchase advances, securities transactions and bank external positions remain separate from income. Financing is not inferred from the subtotal.</x:v>
       </x:c>
       <x:c r="C20" s="2"/>
       <x:c r="D20" s="10" t="str">
         <x:v>Land Commission reports and bank balance sheets for matched dates.</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="80" customHeight="1">
+    <x:row r="21" ht="64" customHeight="1">
       <x:c r="A21" s="10" t="str">
-        <x:v>Adoption rule</x:v>
+        <x:v>Reading the estimate</x:v>
       </x:c>
       <x:c r="B21" s="10" t="str">
-        <x:v>Populate the account only after recording year, territorial coverage, units, source and overlaps. The account may use explicit proxies, but none is silently substituted. Net worker cash and the fiscal grouping are historical working aggregates, not single modern BoP categories.</x:v>
+        <x:v>A sum of included flows, not a complete current account. Unmeasured entries are omitted, not observed zeros. Sandbox alternatives do not change adopted inputs.</x:v>
       </x:c>
       <x:c r="C21" s="2"/>
       <x:c r="D21" s="10" t="str">
         <x:v>Research convention for this workbook.</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="80" customHeight="1">
+    <x:row r="22" ht="64" customHeight="1">
       <x:c r="A22" s="10" t="str">
-        <x:v>Source access</x:v>
+        <x:v>Sources</x:v>
       </x:c>
       <x:c r="B22" s="10" t="str">
-        <x:v>HNAG spreadsheet inspected locally; online texts and transcriptions inspected. Several original scans and revised-series checks remain outstanding. This first assembly is not a complete measured balance of payments.</x:v>
+        <x:v>Evidence lists inputs and references. Supporting schedules preserve original values, calculations, alternatives and unresolved coverage issues.</x:v>
       </x:c>
       <x:c r="C22" s="2"/>
       <x:c r="D22" s="10" t="str">
-        <x:v>Evidence register records the source behind each numeric input.</x:v>
+        <x:v>See Evidence and the component schedules.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="23" customHeight="1">
@@ -31629,7 +31629,7 @@
         <x:v>Predecessors and interpretation</x:v>
       </x:c>
       <x:c r="B32" s="47" t="str">
-        <x:v>Review of 13 October 2026; adopted figures unchanged.</x:v>
+        <x:v>Historical comparisons; source estimates remain distinct from adopted inputs.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="115" customHeight="1">
@@ -31709,7 +31709,7 @@
         <x:v>Priorities</x:v>
       </x:c>
       <x:c r="B42" s="48" t="str">
-        <x:v>Reconcile institutional investment earnings and outward profits; reconcile imperial-service receipts by residence; retrieve paired revised 1904 trade totals. Keep £5m rents and £250,000 seasonal earnings as adopted. Missing flows are omitted, not measured zero; the subtotal does not establish financial-account financing.</x:v>
+        <x:v>Remaining gaps: institutional investment earnings and outward profits; imperial-service receipts by residence; transport, insurance and travel. Trade inputs remain the adopted Kennedy/CEPH/HNAG series.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>